<commit_message>
chore(gransuelo): actualizar plantilla con modificacion de las 17:58
</commit_message>
<xml_diff>
--- a/app/templates/informes/GranSuelo/1-INF.-N-000-26-SU24-GRA.-S.-V09.xlsx
+++ b/app/templates/informes/GranSuelo/1-INF.-N-000-26-SU24-GRA.-S.-V09.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\GranSuelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A50C744-50D6-4346-A072-05BFD129E348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF801408-7953-48AA-B302-714A567FF554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2760" yWindow="1320" windowWidth="20280" windowHeight="10920" tabRatio="547" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="547" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="99" r:id="rId1"/>
@@ -7948,6 +7948,80 @@
     <xf numFmtId="179" fontId="4" fillId="3" borderId="99" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="99" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="77" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="97" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="105" fillId="0" borderId="77" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="105" fillId="0" borderId="95" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="105" fillId="0" borderId="97" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="155" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="157" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
@@ -7956,6 +8030,42 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="105" fillId="0" borderId="77" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="105" fillId="0" borderId="95" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="105" fillId="0" borderId="97" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="83" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="84" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="155" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="157" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="77" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -7975,12 +8085,6 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="77" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="97" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="97" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -8005,15 +8109,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="105" fillId="0" borderId="77" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="105" fillId="0" borderId="95" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="105" fillId="0" borderId="97" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -8023,100 +8118,217 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="155" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="157" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="161" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="162" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="105" fillId="0" borderId="77" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="105" fillId="0" borderId="95" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="105" fillId="0" borderId="97" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="163" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="158" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="159" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="160" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="99" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="83" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="158" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="160" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="84" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="155" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="157" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="99" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="12" fontId="17" fillId="0" borderId="99" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="77" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="118" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="155" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="156" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="157" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="25" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="161" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="163" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="161" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="163" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="17" fillId="0" borderId="161" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="17" fillId="0" borderId="163" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="77" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="90" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="148" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="161" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="163" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="164" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="166" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="165" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="188" fontId="17" fillId="0" borderId="86" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -8139,218 +8351,6 @@
     <xf numFmtId="12" fontId="17" fillId="0" borderId="163" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="161" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="163" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="161" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="162" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="163" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="17" fillId="0" borderId="161" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="17" fillId="0" borderId="163" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="0" borderId="161" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="0" borderId="163" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="99" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="77" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="90" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="148" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="161" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="163" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="164" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="166" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="165" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="77" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="118" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="155" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="156" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="157" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="185" fontId="25" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="12" fontId="17" fillId="0" borderId="99" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="158" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="159" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="160" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="97" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="0" borderId="158" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="0" borderId="160" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="183" fontId="4" fillId="3" borderId="77" xfId="4" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -8454,6 +8454,78 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="56" fillId="3" borderId="130" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="55" fillId="3" borderId="77" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="55" fillId="3" borderId="95" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="55" fillId="3" borderId="97" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="56" fillId="3" borderId="77" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="56" fillId="3" borderId="97" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="83" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="84" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="86" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="54" fillId="3" borderId="77" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="54" fillId="3" borderId="95" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="54" fillId="3" borderId="96" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="54" fillId="3" borderId="1" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -8470,77 +8542,62 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="101" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="83" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="84" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="86" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="11" borderId="79" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="47" fillId="11" borderId="80" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="12" borderId="82" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="12" borderId="74" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="12" borderId="91" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="83" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="84" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="86" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="14" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="16" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="13" borderId="83" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="54" fillId="3" borderId="77" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="54" fillId="3" borderId="95" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="54" fillId="3" borderId="96" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="54" fillId="3" borderId="1" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="55" fillId="3" borderId="77" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="55" fillId="3" borderId="95" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="55" fillId="3" borderId="97" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="56" fillId="3" borderId="77" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="56" fillId="3" borderId="97" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="21" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="50" fillId="13" borderId="85" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="13" borderId="87" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="13" borderId="88" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="10" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="6" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -8592,63 +8649,6 @@
     </xf>
     <xf numFmtId="0" fontId="47" fillId="11" borderId="78" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="101" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="11" borderId="79" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="11" borderId="80" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="82" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="74" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="91" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="12" borderId="83" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="12" borderId="84" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="12" borderId="86" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="12" borderId="14" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="12" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="12" borderId="16" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="83" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="85" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="87" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="88" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="12" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="12" borderId="10" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="9" borderId="68" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -21606,38 +21606,38 @@
       <c r="O6" s="760"/>
     </row>
     <row r="7" spans="1:21" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="782" t="s">
+      <c r="A7" s="814" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="782"/>
-      <c r="C7" s="782"/>
-      <c r="D7" s="782"/>
-      <c r="E7" s="782"/>
-      <c r="F7" s="782"/>
-      <c r="G7" s="782"/>
-      <c r="H7" s="782"/>
-      <c r="I7" s="782"/>
-      <c r="J7" s="782"/>
-      <c r="K7" s="782"/>
+      <c r="B7" s="814"/>
+      <c r="C7" s="814"/>
+      <c r="D7" s="814"/>
+      <c r="E7" s="814"/>
+      <c r="F7" s="814"/>
+      <c r="G7" s="814"/>
+      <c r="H7" s="814"/>
+      <c r="I7" s="814"/>
+      <c r="J7" s="814"/>
+      <c r="K7" s="814"/>
       <c r="N7" s="291" t="s">
         <v>447</v>
       </c>
       <c r="O7" s="760"/>
     </row>
     <row r="8" spans="1:21" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="783" t="s">
+      <c r="A8" s="815" t="s">
         <v>477</v>
       </c>
-      <c r="B8" s="783"/>
-      <c r="C8" s="783"/>
-      <c r="D8" s="783"/>
-      <c r="E8" s="783"/>
-      <c r="F8" s="783"/>
-      <c r="G8" s="783"/>
-      <c r="H8" s="783"/>
-      <c r="I8" s="783"/>
-      <c r="J8" s="783"/>
-      <c r="K8" s="783"/>
+      <c r="B8" s="815"/>
+      <c r="C8" s="815"/>
+      <c r="D8" s="815"/>
+      <c r="E8" s="815"/>
+      <c r="F8" s="815"/>
+      <c r="G8" s="815"/>
+      <c r="H8" s="815"/>
+      <c r="I8" s="815"/>
+      <c r="J8" s="815"/>
+      <c r="K8" s="815"/>
       <c r="N8" s="291" t="s">
         <v>550</v>
       </c>
@@ -21663,18 +21663,18 @@
     <row r="10" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="485"/>
       <c r="C10" s="485"/>
-      <c r="D10" s="784" t="s">
+      <c r="D10" s="816" t="s">
         <v>478</v>
       </c>
-      <c r="E10" s="785"/>
-      <c r="F10" s="784" t="s">
+      <c r="E10" s="817"/>
+      <c r="F10" s="816" t="s">
         <v>479</v>
       </c>
-      <c r="G10" s="785"/>
-      <c r="H10" s="784" t="s">
+      <c r="G10" s="817"/>
+      <c r="H10" s="816" t="s">
         <v>30</v>
       </c>
-      <c r="I10" s="785"/>
+      <c r="I10" s="817"/>
       <c r="J10" s="679" t="s">
         <v>467</v>
       </c>
@@ -21688,12 +21688,12 @@
       <c r="A11" s="485"/>
       <c r="B11" s="485"/>
       <c r="C11" s="485"/>
-      <c r="D11" s="786"/>
-      <c r="E11" s="787"/>
-      <c r="F11" s="786"/>
-      <c r="G11" s="787"/>
-      <c r="H11" s="786"/>
-      <c r="I11" s="787"/>
+      <c r="D11" s="779"/>
+      <c r="E11" s="780"/>
+      <c r="F11" s="779"/>
+      <c r="G11" s="780"/>
+      <c r="H11" s="779"/>
+      <c r="I11" s="780"/>
       <c r="J11" s="682"/>
       <c r="K11" s="386"/>
       <c r="L11" s="681"/>
@@ -21723,19 +21723,19 @@
       <c r="O12" s="761"/>
     </row>
     <row r="13" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="788" t="s">
+      <c r="A13" s="818" t="s">
         <v>480</v>
       </c>
-      <c r="B13" s="789"/>
-      <c r="C13" s="789"/>
-      <c r="D13" s="789"/>
-      <c r="E13" s="789"/>
-      <c r="F13" s="789"/>
-      <c r="G13" s="789"/>
-      <c r="H13" s="789"/>
-      <c r="I13" s="789"/>
-      <c r="J13" s="789"/>
-      <c r="K13" s="790"/>
+      <c r="B13" s="819"/>
+      <c r="C13" s="819"/>
+      <c r="D13" s="819"/>
+      <c r="E13" s="819"/>
+      <c r="F13" s="819"/>
+      <c r="G13" s="819"/>
+      <c r="H13" s="819"/>
+      <c r="I13" s="819"/>
+      <c r="J13" s="819"/>
+      <c r="K13" s="820"/>
       <c r="L13" s="681"/>
       <c r="M13" s="681"/>
       <c r="N13" s="291" t="s">
@@ -21744,19 +21744,19 @@
       <c r="O13" s="761"/>
     </row>
     <row r="14" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="791" t="s">
+      <c r="A14" s="821" t="s">
         <v>481</v>
       </c>
-      <c r="B14" s="792"/>
-      <c r="C14" s="792"/>
-      <c r="D14" s="792"/>
-      <c r="E14" s="792"/>
-      <c r="F14" s="792"/>
-      <c r="G14" s="792"/>
-      <c r="H14" s="792"/>
-      <c r="I14" s="792"/>
-      <c r="J14" s="792"/>
-      <c r="K14" s="793"/>
+      <c r="B14" s="822"/>
+      <c r="C14" s="822"/>
+      <c r="D14" s="822"/>
+      <c r="E14" s="822"/>
+      <c r="F14" s="822"/>
+      <c r="G14" s="822"/>
+      <c r="H14" s="822"/>
+      <c r="I14" s="822"/>
+      <c r="J14" s="822"/>
+      <c r="K14" s="823"/>
       <c r="L14" s="681"/>
       <c r="M14" s="681"/>
       <c r="N14" s="759"/>
@@ -21776,21 +21776,21 @@
       <c r="U15" s="684"/>
     </row>
     <row r="16" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="794" t="s">
+      <c r="A16" s="804" t="s">
         <v>482</v>
       </c>
-      <c r="B16" s="795"/>
-      <c r="C16" s="796"/>
-      <c r="E16" s="797" t="s">
+      <c r="B16" s="805"/>
+      <c r="C16" s="806"/>
+      <c r="E16" s="824" t="s">
         <v>372</v>
       </c>
-      <c r="F16" s="798"/>
-      <c r="G16" s="798"/>
-      <c r="H16" s="799"/>
-      <c r="J16" s="794" t="s">
+      <c r="F16" s="825"/>
+      <c r="G16" s="825"/>
+      <c r="H16" s="826"/>
+      <c r="J16" s="804" t="s">
         <v>483</v>
       </c>
-      <c r="K16" s="796"/>
+      <c r="K16" s="806"/>
       <c r="M16" s="684"/>
       <c r="N16" s="291" t="s">
         <v>245</v>
@@ -21806,16 +21806,16 @@
       <c r="A17" s="687" t="s">
         <v>484</v>
       </c>
-      <c r="B17" s="778"/>
-      <c r="C17" s="779"/>
+      <c r="B17" s="799"/>
+      <c r="C17" s="800"/>
       <c r="E17" s="688" t="s">
         <v>485</v>
       </c>
       <c r="F17" s="689"/>
       <c r="G17" s="690"/>
       <c r="H17" s="691"/>
-      <c r="J17" s="780"/>
-      <c r="K17" s="781"/>
+      <c r="J17" s="812"/>
+      <c r="K17" s="813"/>
       <c r="M17" s="684"/>
       <c r="N17" s="291" t="s">
         <v>552</v>
@@ -21831,8 +21831,8 @@
       <c r="A18" s="687" t="s">
         <v>486</v>
       </c>
-      <c r="B18" s="778"/>
-      <c r="C18" s="779"/>
+      <c r="B18" s="799"/>
+      <c r="C18" s="800"/>
       <c r="E18" s="688" t="s">
         <v>487</v>
       </c>
@@ -21855,10 +21855,10 @@
       <c r="F19" s="689"/>
       <c r="G19" s="690"/>
       <c r="H19" s="694"/>
-      <c r="J19" s="804" t="s">
+      <c r="J19" s="782" t="s">
         <v>489</v>
       </c>
-      <c r="K19" s="805"/>
+      <c r="K19" s="783"/>
       <c r="M19" s="684"/>
       <c r="N19" s="692"/>
       <c r="O19" s="685"/>
@@ -21869,11 +21869,11 @@
       <c r="U19" s="686"/>
     </row>
     <row r="20" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="806" t="s">
+      <c r="A20" s="789" t="s">
         <v>490</v>
       </c>
-      <c r="B20" s="807"/>
-      <c r="C20" s="808"/>
+      <c r="B20" s="790"/>
+      <c r="C20" s="791"/>
       <c r="E20" s="695" t="s">
         <v>491</v>
       </c>
@@ -21897,8 +21897,8 @@
       <c r="A21" s="687" t="s">
         <v>492</v>
       </c>
-      <c r="B21" s="809"/>
-      <c r="C21" s="810"/>
+      <c r="B21" s="801"/>
+      <c r="C21" s="802"/>
       <c r="E21" s="700"/>
       <c r="F21" s="700"/>
       <c r="G21" s="700"/>
@@ -21919,14 +21919,14 @@
       <c r="A22" s="687" t="s">
         <v>494</v>
       </c>
-      <c r="B22" s="809"/>
-      <c r="C22" s="810"/>
-      <c r="E22" s="804" t="s">
+      <c r="B22" s="801"/>
+      <c r="C22" s="802"/>
+      <c r="E22" s="782" t="s">
         <v>369</v>
       </c>
-      <c r="F22" s="811"/>
-      <c r="G22" s="811"/>
-      <c r="H22" s="805"/>
+      <c r="F22" s="803"/>
+      <c r="G22" s="803"/>
+      <c r="H22" s="783"/>
       <c r="I22" s="701"/>
       <c r="J22" s="486" t="s">
         <v>370</v>
@@ -21962,11 +21962,11 @@
       <c r="U23" s="686"/>
     </row>
     <row r="24" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="794" t="s">
+      <c r="A24" s="804" t="s">
         <v>497</v>
       </c>
-      <c r="B24" s="795"/>
-      <c r="C24" s="796"/>
+      <c r="B24" s="805"/>
+      <c r="C24" s="806"/>
       <c r="E24" s="688" t="s">
         <v>498</v>
       </c>
@@ -22118,8 +22118,8 @@
       <c r="A31" s="705" t="s">
         <v>510</v>
       </c>
-      <c r="B31" s="812"/>
-      <c r="C31" s="812"/>
+      <c r="B31" s="807"/>
+      <c r="C31" s="807"/>
       <c r="E31" s="688" t="s">
         <v>511</v>
       </c>
@@ -22142,8 +22142,8 @@
       <c r="A32" s="705" t="s">
         <v>512</v>
       </c>
-      <c r="B32" s="812"/>
-      <c r="C32" s="812"/>
+      <c r="B32" s="807"/>
+      <c r="C32" s="807"/>
       <c r="E32" s="688" t="s">
         <v>513</v>
       </c>
@@ -22182,17 +22182,17 @@
       <c r="U33" s="686"/>
     </row>
     <row r="34" spans="1:21" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="806" t="s">
+      <c r="A34" s="789" t="s">
         <v>515</v>
       </c>
-      <c r="B34" s="807"/>
-      <c r="C34" s="808"/>
-      <c r="E34" s="813" t="s">
+      <c r="B34" s="790"/>
+      <c r="C34" s="791"/>
+      <c r="E34" s="808" t="s">
         <v>516</v>
       </c>
-      <c r="F34" s="814"/>
-      <c r="G34" s="800"/>
-      <c r="H34" s="801"/>
+      <c r="F34" s="809"/>
+      <c r="G34" s="795"/>
+      <c r="H34" s="796"/>
       <c r="I34" s="717"/>
       <c r="J34" s="718" t="s">
         <v>517</v>
@@ -22212,10 +22212,10 @@
       </c>
       <c r="B35" s="700"/>
       <c r="C35" s="721"/>
-      <c r="E35" s="815"/>
-      <c r="F35" s="816"/>
-      <c r="G35" s="802"/>
-      <c r="H35" s="803"/>
+      <c r="E35" s="810"/>
+      <c r="F35" s="811"/>
+      <c r="G35" s="797"/>
+      <c r="H35" s="798"/>
       <c r="J35" s="722" t="s">
         <v>519</v>
       </c>
@@ -22239,19 +22239,19 @@
       <c r="P36" s="684"/>
     </row>
     <row r="37" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="806" t="s">
+      <c r="A37" s="789" t="s">
         <v>520</v>
       </c>
-      <c r="B37" s="807"/>
-      <c r="C37" s="808"/>
-      <c r="E37" s="824" t="s">
+      <c r="B37" s="790"/>
+      <c r="C37" s="791"/>
+      <c r="E37" s="792" t="s">
         <v>521</v>
       </c>
-      <c r="F37" s="825"/>
-      <c r="G37" s="825"/>
-      <c r="H37" s="825"/>
-      <c r="I37" s="826"/>
-      <c r="K37" s="817" t="s">
+      <c r="F37" s="793"/>
+      <c r="G37" s="793"/>
+      <c r="H37" s="793"/>
+      <c r="I37" s="794"/>
+      <c r="K37" s="778" t="s">
         <v>522</v>
       </c>
       <c r="L37" s="681"/>
@@ -22264,15 +22264,15 @@
       <c r="E38" s="730" t="s">
         <v>548</v>
       </c>
-      <c r="F38" s="786" t="s">
+      <c r="F38" s="779" t="s">
         <v>523</v>
       </c>
-      <c r="G38" s="787"/>
-      <c r="H38" s="786" t="s">
+      <c r="G38" s="780"/>
+      <c r="H38" s="779" t="s">
         <v>524</v>
       </c>
-      <c r="I38" s="787"/>
-      <c r="K38" s="817"/>
+      <c r="I38" s="780"/>
+      <c r="K38" s="778"/>
       <c r="L38" s="681"/>
     </row>
     <row r="39" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -22291,10 +22291,10 @@
       <c r="C40" s="733" t="s">
         <v>526</v>
       </c>
-      <c r="D40" s="804" t="s">
+      <c r="D40" s="782" t="s">
         <v>527</v>
       </c>
-      <c r="E40" s="805"/>
+      <c r="E40" s="783"/>
       <c r="I40" s="734" t="s">
         <v>528</v>
       </c>
@@ -22307,10 +22307,10 @@
       <c r="C41" s="733" t="s">
         <v>530</v>
       </c>
-      <c r="D41" s="804" t="s">
+      <c r="D41" s="782" t="s">
         <v>366</v>
       </c>
-      <c r="E41" s="805"/>
+      <c r="E41" s="783"/>
       <c r="J41" s="735"/>
       <c r="L41" s="681"/>
     </row>
@@ -22417,14 +22417,14 @@
       </c>
       <c r="D50" s="738"/>
       <c r="E50" s="745"/>
-      <c r="G50" s="819" t="s">
+      <c r="G50" s="784" t="s">
         <v>538</v>
       </c>
-      <c r="H50" s="820"/>
-      <c r="I50" s="819" t="s">
+      <c r="H50" s="785"/>
+      <c r="I50" s="784" t="s">
         <v>539</v>
       </c>
-      <c r="J50" s="820"/>
+      <c r="J50" s="785"/>
       <c r="L50" s="681"/>
       <c r="M50" s="681"/>
     </row>
@@ -22441,8 +22441,8 @@
         <v>540</v>
       </c>
       <c r="H51" s="747"/>
-      <c r="I51" s="821"/>
-      <c r="J51" s="822"/>
+      <c r="I51" s="786"/>
+      <c r="J51" s="787"/>
       <c r="L51" s="681"/>
       <c r="M51" s="681"/>
     </row>
@@ -22459,8 +22459,8 @@
         <v>542</v>
       </c>
       <c r="H52" s="747"/>
-      <c r="I52" s="821"/>
-      <c r="J52" s="822"/>
+      <c r="I52" s="786"/>
+      <c r="J52" s="787"/>
       <c r="L52" s="681"/>
       <c r="M52" s="681"/>
     </row>
@@ -22590,12 +22590,12 @@
       <c r="B62" s="485"/>
       <c r="C62" s="485"/>
       <c r="D62" s="485"/>
-      <c r="E62" s="823"/>
-      <c r="F62" s="823"/>
-      <c r="G62" s="823"/>
-      <c r="H62" s="823"/>
-      <c r="I62" s="823"/>
-      <c r="J62" s="823"/>
+      <c r="E62" s="788"/>
+      <c r="F62" s="788"/>
+      <c r="G62" s="788"/>
+      <c r="H62" s="788"/>
+      <c r="I62" s="788"/>
+      <c r="J62" s="788"/>
       <c r="K62" s="740"/>
       <c r="L62" s="681"/>
       <c r="M62" s="681"/>
@@ -22622,19 +22622,19 @@
       <c r="G64" s="260"/>
     </row>
     <row r="65" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="818" t="s">
+      <c r="A65" s="781" t="s">
         <v>547</v>
       </c>
-      <c r="B65" s="818"/>
-      <c r="C65" s="818"/>
-      <c r="D65" s="818"/>
-      <c r="E65" s="818"/>
-      <c r="F65" s="818"/>
-      <c r="G65" s="818"/>
-      <c r="H65" s="818"/>
-      <c r="I65" s="818"/>
-      <c r="J65" s="818"/>
-      <c r="K65" s="818"/>
+      <c r="B65" s="781"/>
+      <c r="C65" s="781"/>
+      <c r="D65" s="781"/>
+      <c r="E65" s="781"/>
+      <c r="F65" s="781"/>
+      <c r="G65" s="781"/>
+      <c r="H65" s="781"/>
+      <c r="I65" s="781"/>
+      <c r="J65" s="781"/>
+      <c r="K65" s="781"/>
     </row>
     <row r="66" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -22645,32 +22645,6 @@
     <protectedRange sqref="C10:C11 C62" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="41">
-    <mergeCell ref="K37:K38"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="A65:K65"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="G50:H50"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="I52:J52"/>
-    <mergeCell ref="E62:G62"/>
-    <mergeCell ref="H62:J62"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="E37:I37"/>
-    <mergeCell ref="G34:H35"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="E22:H22"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="E34:F35"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="J17:K17"/>
     <mergeCell ref="A7:K7"/>
@@ -22686,6 +22660,32 @@
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="E16:H16"/>
     <mergeCell ref="J16:K16"/>
+    <mergeCell ref="G34:H35"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="E22:H22"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="E34:F35"/>
+    <mergeCell ref="K37:K38"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="A65:K65"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="G50:H50"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="I52:J52"/>
+    <mergeCell ref="E62:G62"/>
+    <mergeCell ref="H62:J62"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="E37:I37"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0.39370078740157483" bottom="0" header="0" footer="0"/>
@@ -22850,14 +22850,14 @@
       <c r="L5" s="564"/>
       <c r="M5" s="564"/>
       <c r="N5" s="564"/>
-      <c r="Q5" s="872" t="s">
+      <c r="Q5" s="844" t="s">
         <v>369</v>
       </c>
-      <c r="R5" s="873"/>
-      <c r="S5" s="873"/>
-      <c r="T5" s="873"/>
-      <c r="U5" s="873"/>
-      <c r="V5" s="874"/>
+      <c r="R5" s="845"/>
+      <c r="S5" s="845"/>
+      <c r="T5" s="845"/>
+      <c r="U5" s="845"/>
+      <c r="V5" s="846"/>
       <c r="X5" s="474" t="s">
         <v>370</v>
       </c>
@@ -22918,22 +22918,22 @@
       </c>
     </row>
     <row r="7" spans="1:30" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="782" t="s">
+      <c r="A7" s="814" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="782"/>
-      <c r="C7" s="782"/>
-      <c r="D7" s="782"/>
-      <c r="E7" s="782"/>
-      <c r="F7" s="782"/>
-      <c r="G7" s="782"/>
-      <c r="H7" s="782"/>
-      <c r="I7" s="782"/>
-      <c r="J7" s="782"/>
-      <c r="K7" s="782"/>
-      <c r="L7" s="782"/>
-      <c r="M7" s="782"/>
-      <c r="N7" s="782"/>
+      <c r="B7" s="814"/>
+      <c r="C7" s="814"/>
+      <c r="D7" s="814"/>
+      <c r="E7" s="814"/>
+      <c r="F7" s="814"/>
+      <c r="G7" s="814"/>
+      <c r="H7" s="814"/>
+      <c r="I7" s="814"/>
+      <c r="J7" s="814"/>
+      <c r="K7" s="814"/>
+      <c r="L7" s="814"/>
+      <c r="M7" s="814"/>
+      <c r="N7" s="814"/>
       <c r="Q7" s="478" t="s">
         <v>422</v>
       </c>
@@ -22972,22 +22972,22 @@
       </c>
     </row>
     <row r="8" spans="1:30" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="884">
+      <c r="A8" s="856">
         <v>0</v>
       </c>
-      <c r="B8" s="884"/>
-      <c r="C8" s="884"/>
-      <c r="D8" s="884"/>
-      <c r="E8" s="884"/>
-      <c r="F8" s="884"/>
-      <c r="G8" s="884"/>
-      <c r="H8" s="884"/>
-      <c r="I8" s="884"/>
-      <c r="J8" s="884"/>
-      <c r="K8" s="884"/>
-      <c r="L8" s="884"/>
-      <c r="M8" s="884"/>
-      <c r="N8" s="884"/>
+      <c r="B8" s="856"/>
+      <c r="C8" s="856"/>
+      <c r="D8" s="856"/>
+      <c r="E8" s="856"/>
+      <c r="F8" s="856"/>
+      <c r="G8" s="856"/>
+      <c r="H8" s="856"/>
+      <c r="I8" s="856"/>
+      <c r="J8" s="856"/>
+      <c r="K8" s="856"/>
+      <c r="L8" s="856"/>
+      <c r="M8" s="856"/>
+      <c r="N8" s="856"/>
       <c r="Q8" s="478" t="s">
         <v>423</v>
       </c>
@@ -23032,18 +23032,18 @@
       <c r="B9" s="287" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="886">
+      <c r="C9" s="858">
         <f>+FORMATO!O2</f>
         <v>0</v>
       </c>
-      <c r="D9" s="886"/>
-      <c r="E9" s="886"/>
-      <c r="F9" s="886"/>
-      <c r="G9" s="886"/>
-      <c r="H9" s="886"/>
-      <c r="I9" s="886"/>
-      <c r="J9" s="886"/>
-      <c r="K9" s="886"/>
+      <c r="D9" s="858"/>
+      <c r="E9" s="858"/>
+      <c r="F9" s="858"/>
+      <c r="G9" s="858"/>
+      <c r="H9" s="858"/>
+      <c r="I9" s="858"/>
+      <c r="J9" s="858"/>
+      <c r="K9" s="858"/>
       <c r="L9" s="289" t="s">
         <v>31</v>
       </c>
@@ -23088,18 +23088,18 @@
       <c r="B10" s="288" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="886">
+      <c r="C10" s="858">
         <f>+FORMATO!O3</f>
         <v>0</v>
       </c>
-      <c r="D10" s="886"/>
-      <c r="E10" s="886"/>
-      <c r="F10" s="886"/>
-      <c r="G10" s="886"/>
-      <c r="H10" s="886"/>
-      <c r="I10" s="886"/>
-      <c r="J10" s="886"/>
-      <c r="K10" s="886"/>
+      <c r="D10" s="858"/>
+      <c r="E10" s="858"/>
+      <c r="F10" s="858"/>
+      <c r="G10" s="858"/>
+      <c r="H10" s="858"/>
+      <c r="I10" s="858"/>
+      <c r="J10" s="858"/>
+      <c r="K10" s="858"/>
       <c r="L10" s="764" t="s">
         <v>447</v>
       </c>
@@ -23127,18 +23127,18 @@
       <c r="B11" s="288" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="886">
+      <c r="C11" s="858">
         <f>+FORMATO!O4</f>
         <v>0</v>
       </c>
-      <c r="D11" s="886"/>
-      <c r="E11" s="886"/>
-      <c r="F11" s="886"/>
-      <c r="G11" s="886"/>
-      <c r="H11" s="886"/>
-      <c r="I11" s="886"/>
-      <c r="J11" s="886"/>
-      <c r="K11" s="886"/>
+      <c r="D11" s="858"/>
+      <c r="E11" s="858"/>
+      <c r="F11" s="858"/>
+      <c r="G11" s="858"/>
+      <c r="H11" s="858"/>
+      <c r="I11" s="858"/>
+      <c r="J11" s="858"/>
+      <c r="K11" s="858"/>
       <c r="L11" s="291" t="s">
         <v>466</v>
       </c>
@@ -23151,14 +23151,14 @@
       </c>
       <c r="O11" s="570"/>
       <c r="P11" s="570"/>
-      <c r="Q11" s="875" t="s">
+      <c r="Q11" s="847" t="s">
         <v>40</v>
       </c>
-      <c r="R11" s="885"/>
-      <c r="S11" s="885"/>
-      <c r="T11" s="885"/>
-      <c r="U11" s="885"/>
-      <c r="V11" s="876"/>
+      <c r="R11" s="857"/>
+      <c r="S11" s="857"/>
+      <c r="T11" s="857"/>
+      <c r="U11" s="857"/>
+      <c r="V11" s="848"/>
       <c r="X11" s="571" t="s">
         <v>198</v>
       </c>
@@ -23179,18 +23179,18 @@
       <c r="B12" s="288" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="886">
+      <c r="C12" s="858">
         <f>+FORMATO!O5</f>
         <v>0</v>
       </c>
-      <c r="D12" s="886"/>
-      <c r="E12" s="886"/>
-      <c r="F12" s="886"/>
-      <c r="G12" s="886"/>
-      <c r="H12" s="886"/>
-      <c r="I12" s="886"/>
-      <c r="J12" s="886"/>
-      <c r="K12" s="886"/>
+      <c r="D12" s="858"/>
+      <c r="E12" s="858"/>
+      <c r="F12" s="858"/>
+      <c r="G12" s="858"/>
+      <c r="H12" s="858"/>
+      <c r="I12" s="858"/>
+      <c r="J12" s="858"/>
+      <c r="K12" s="858"/>
       <c r="L12" s="764" t="s">
         <v>253</v>
       </c>
@@ -23276,22 +23276,22 @@
       </c>
     </row>
     <row r="14" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="877" t="s">
+      <c r="A14" s="849" t="s">
         <v>250</v>
       </c>
-      <c r="B14" s="878"/>
-      <c r="C14" s="878"/>
-      <c r="D14" s="879"/>
-      <c r="E14" s="878"/>
-      <c r="F14" s="879"/>
-      <c r="G14" s="879"/>
-      <c r="H14" s="879"/>
-      <c r="I14" s="879"/>
-      <c r="J14" s="879"/>
-      <c r="K14" s="879"/>
-      <c r="L14" s="879"/>
-      <c r="M14" s="879"/>
-      <c r="N14" s="880"/>
+      <c r="B14" s="850"/>
+      <c r="C14" s="850"/>
+      <c r="D14" s="851"/>
+      <c r="E14" s="850"/>
+      <c r="F14" s="851"/>
+      <c r="G14" s="851"/>
+      <c r="H14" s="851"/>
+      <c r="I14" s="851"/>
+      <c r="J14" s="851"/>
+      <c r="K14" s="851"/>
+      <c r="L14" s="851"/>
+      <c r="M14" s="851"/>
+      <c r="N14" s="852"/>
       <c r="O14" s="570"/>
       <c r="P14" s="570"/>
       <c r="Q14" s="478" t="s">
@@ -23322,22 +23322,22 @@
       </c>
     </row>
     <row r="15" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="881" t="s">
+      <c r="A15" s="853" t="s">
         <v>476</v>
       </c>
-      <c r="B15" s="882"/>
-      <c r="C15" s="882"/>
-      <c r="D15" s="882"/>
-      <c r="E15" s="882"/>
-      <c r="F15" s="882"/>
-      <c r="G15" s="882"/>
-      <c r="H15" s="882"/>
-      <c r="I15" s="882"/>
-      <c r="J15" s="882"/>
-      <c r="K15" s="882"/>
-      <c r="L15" s="882"/>
-      <c r="M15" s="882"/>
-      <c r="N15" s="883"/>
+      <c r="B15" s="854"/>
+      <c r="C15" s="854"/>
+      <c r="D15" s="854"/>
+      <c r="E15" s="854"/>
+      <c r="F15" s="854"/>
+      <c r="G15" s="854"/>
+      <c r="H15" s="854"/>
+      <c r="I15" s="854"/>
+      <c r="J15" s="854"/>
+      <c r="K15" s="854"/>
+      <c r="L15" s="854"/>
+      <c r="M15" s="854"/>
+      <c r="N15" s="855"/>
       <c r="O15" s="570"/>
       <c r="P15" s="570"/>
       <c r="V15" s="386"/>
@@ -23369,14 +23369,14 @@
       <c r="N16" s="298"/>
       <c r="O16" s="570"/>
       <c r="P16" s="570"/>
-      <c r="Q16" s="875" t="s">
+      <c r="Q16" s="847" t="s">
         <v>438</v>
       </c>
-      <c r="R16" s="885"/>
-      <c r="S16" s="885"/>
-      <c r="T16" s="885"/>
-      <c r="U16" s="885"/>
-      <c r="V16" s="876"/>
+      <c r="R16" s="857"/>
+      <c r="S16" s="857"/>
+      <c r="T16" s="857"/>
+      <c r="U16" s="857"/>
+      <c r="V16" s="848"/>
       <c r="W16" s="578"/>
     </row>
     <row r="17" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -23411,12 +23411,12 @@
         <f>U17+(U17*$Z$14)</f>
         <v>0</v>
       </c>
-      <c r="X17" s="857" t="s">
+      <c r="X17" s="865" t="s">
         <v>433</v>
       </c>
-      <c r="Y17" s="858"/>
-      <c r="Z17" s="858"/>
-      <c r="AA17" s="859"/>
+      <c r="Y17" s="866"/>
+      <c r="Z17" s="866"/>
+      <c r="AA17" s="867"/>
       <c r="AB17" s="599" t="s">
         <v>441</v>
       </c>
@@ -23645,15 +23645,15 @@
       <c r="B23" s="621"/>
       <c r="C23" s="621"/>
       <c r="D23" s="621"/>
-      <c r="E23" s="862" t="s">
+      <c r="E23" s="870" t="s">
         <v>448</v>
       </c>
-      <c r="F23" s="868"/>
-      <c r="G23" s="868"/>
-      <c r="H23" s="868"/>
-      <c r="I23" s="868"/>
-      <c r="J23" s="863"/>
-      <c r="K23" s="860" t="s">
+      <c r="F23" s="876"/>
+      <c r="G23" s="876"/>
+      <c r="H23" s="876"/>
+      <c r="I23" s="876"/>
+      <c r="J23" s="871"/>
+      <c r="K23" s="868" t="s">
         <v>385</v>
       </c>
       <c r="L23" s="621"/>
@@ -23661,10 +23661,10 @@
       <c r="N23" s="307"/>
       <c r="O23" s="570"/>
       <c r="P23" s="583"/>
-      <c r="Q23" s="875" t="s">
+      <c r="Q23" s="847" t="s">
         <v>357</v>
       </c>
-      <c r="R23" s="876"/>
+      <c r="R23" s="848"/>
       <c r="S23" s="387" t="s">
         <v>356</v>
       </c>
@@ -23697,17 +23697,17 @@
       <c r="B24" s="621"/>
       <c r="C24" s="621"/>
       <c r="D24" s="621"/>
-      <c r="E24" s="862" t="s">
+      <c r="E24" s="870" t="s">
         <v>358</v>
       </c>
-      <c r="F24" s="868"/>
-      <c r="G24" s="868"/>
-      <c r="H24" s="863"/>
-      <c r="I24" s="862" t="s">
+      <c r="F24" s="876"/>
+      <c r="G24" s="876"/>
+      <c r="H24" s="871"/>
+      <c r="I24" s="870" t="s">
         <v>457</v>
       </c>
-      <c r="J24" s="863"/>
-      <c r="K24" s="861"/>
+      <c r="J24" s="871"/>
+      <c r="K24" s="869"/>
       <c r="L24" s="621"/>
       <c r="M24" s="631"/>
       <c r="N24" s="307"/>
@@ -23756,16 +23756,16 @@
       <c r="B25" s="623"/>
       <c r="C25" s="623"/>
       <c r="D25" s="623"/>
-      <c r="E25" s="869" t="s">
+      <c r="E25" s="877" t="s">
         <v>350</v>
       </c>
-      <c r="F25" s="870"/>
-      <c r="G25" s="870"/>
-      <c r="H25" s="871"/>
-      <c r="I25" s="864" t="s">
+      <c r="F25" s="878"/>
+      <c r="G25" s="878"/>
+      <c r="H25" s="879"/>
+      <c r="I25" s="872" t="s">
         <v>449</v>
       </c>
-      <c r="J25" s="865"/>
+      <c r="J25" s="873"/>
       <c r="K25" s="617" t="e">
         <f>IF($I$66="Método A",FIXED(($W$25),0),FIXED(($W$25),1))</f>
         <v>#DIV/0!</v>
@@ -23812,16 +23812,16 @@
       <c r="B26" s="623"/>
       <c r="C26" s="623"/>
       <c r="D26" s="623"/>
-      <c r="E26" s="835" t="s">
+      <c r="E26" s="827" t="s">
         <v>351</v>
       </c>
-      <c r="F26" s="836"/>
-      <c r="G26" s="836"/>
-      <c r="H26" s="837"/>
-      <c r="I26" s="866" t="s">
+      <c r="F26" s="828"/>
+      <c r="G26" s="828"/>
+      <c r="H26" s="829"/>
+      <c r="I26" s="874" t="s">
         <v>450</v>
       </c>
-      <c r="J26" s="867"/>
+      <c r="J26" s="875"/>
       <c r="K26" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$26),0),FIXED(($W$26),1))</f>
         <v>#DIV/0!</v>
@@ -23838,7 +23838,7 @@
         <v>50</v>
       </c>
       <c r="S26" s="665">
-        <f>+FORMATO!E43</f>
+        <f>+FORMATO!D43</f>
         <v>0</v>
       </c>
       <c r="T26" s="523">
@@ -23868,16 +23868,16 @@
       <c r="B27" s="624"/>
       <c r="C27" s="624"/>
       <c r="D27" s="624"/>
-      <c r="E27" s="830" t="s">
+      <c r="E27" s="897" t="s">
         <v>353</v>
       </c>
-      <c r="F27" s="831"/>
-      <c r="G27" s="831"/>
-      <c r="H27" s="832"/>
-      <c r="I27" s="833" t="s">
+      <c r="F27" s="898"/>
+      <c r="G27" s="898"/>
+      <c r="H27" s="899"/>
+      <c r="I27" s="861" t="s">
         <v>451</v>
       </c>
-      <c r="J27" s="834"/>
+      <c r="J27" s="862"/>
       <c r="K27" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$27),0),FIXED(($W$27),1))</f>
         <v>#DIV/0!</v>
@@ -23894,7 +23894,7 @@
         <v>37.5</v>
       </c>
       <c r="S27" s="665">
-        <f>+FORMATO!E44</f>
+        <f>+FORMATO!D44</f>
         <v>0</v>
       </c>
       <c r="T27" s="523">
@@ -23924,16 +23924,16 @@
       <c r="B28" s="623"/>
       <c r="C28" s="623"/>
       <c r="D28" s="623"/>
-      <c r="E28" s="835" t="s">
+      <c r="E28" s="827" t="s">
         <v>352</v>
       </c>
-      <c r="F28" s="836"/>
-      <c r="G28" s="836"/>
-      <c r="H28" s="837"/>
-      <c r="I28" s="833" t="s">
+      <c r="F28" s="828"/>
+      <c r="G28" s="828"/>
+      <c r="H28" s="829"/>
+      <c r="I28" s="861" t="s">
         <v>452</v>
       </c>
-      <c r="J28" s="834"/>
+      <c r="J28" s="862"/>
       <c r="K28" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$28),0),FIXED(($W$28),1))</f>
         <v>#DIV/0!</v>
@@ -23950,7 +23950,7 @@
         <v>25</v>
       </c>
       <c r="S28" s="665">
-        <f>+FORMATO!E45</f>
+        <f>+FORMATO!D45</f>
         <v>0</v>
       </c>
       <c r="T28" s="523">
@@ -23980,16 +23980,16 @@
       <c r="B29" s="623"/>
       <c r="C29" s="623"/>
       <c r="D29" s="623"/>
-      <c r="E29" s="835" t="s">
+      <c r="E29" s="827" t="s">
         <v>354</v>
       </c>
-      <c r="F29" s="836"/>
-      <c r="G29" s="836"/>
-      <c r="H29" s="837"/>
-      <c r="I29" s="833" t="s">
+      <c r="F29" s="828"/>
+      <c r="G29" s="828"/>
+      <c r="H29" s="829"/>
+      <c r="I29" s="861" t="s">
         <v>453</v>
       </c>
-      <c r="J29" s="834"/>
+      <c r="J29" s="862"/>
       <c r="K29" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$29),0),FIXED(($W$29),1))</f>
         <v>#DIV/0!</v>
@@ -24006,7 +24006,7 @@
         <v>19</v>
       </c>
       <c r="S29" s="665">
-        <f>+FORMATO!E46</f>
+        <f>+FORMATO!D46</f>
         <v>0</v>
       </c>
       <c r="T29" s="523">
@@ -24036,16 +24036,16 @@
       <c r="B30" s="623"/>
       <c r="C30" s="623"/>
       <c r="D30" s="623"/>
-      <c r="E30" s="835" t="s">
+      <c r="E30" s="827" t="s">
         <v>355</v>
       </c>
-      <c r="F30" s="836"/>
-      <c r="G30" s="836"/>
-      <c r="H30" s="837"/>
-      <c r="I30" s="833" t="s">
+      <c r="F30" s="828"/>
+      <c r="G30" s="828"/>
+      <c r="H30" s="829"/>
+      <c r="I30" s="861" t="s">
         <v>454</v>
       </c>
-      <c r="J30" s="834"/>
+      <c r="J30" s="862"/>
       <c r="K30" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$30),0),FIXED(($W$30),1))</f>
         <v>#DIV/0!</v>
@@ -24062,7 +24062,7 @@
         <v>9.5</v>
       </c>
       <c r="S30" s="665">
-        <f>+FORMATO!E47</f>
+        <f>+FORMATO!D47</f>
         <v>0</v>
       </c>
       <c r="T30" s="523">
@@ -24092,16 +24092,16 @@
       <c r="B31" s="623"/>
       <c r="C31" s="623"/>
       <c r="D31" s="623"/>
-      <c r="E31" s="835" t="s">
+      <c r="E31" s="827" t="s">
         <v>231</v>
       </c>
-      <c r="F31" s="836"/>
-      <c r="G31" s="836"/>
-      <c r="H31" s="837"/>
-      <c r="I31" s="838" t="s">
+      <c r="F31" s="828"/>
+      <c r="G31" s="828"/>
+      <c r="H31" s="829"/>
+      <c r="I31" s="863" t="s">
         <v>455</v>
       </c>
-      <c r="J31" s="839"/>
+      <c r="J31" s="864"/>
       <c r="K31" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$31),0),FIXED(($W$31),1))</f>
         <v>#DIV/0!</v>
@@ -24118,7 +24118,7 @@
         <v>4.75</v>
       </c>
       <c r="S31" s="665">
-        <f>+FORMATO!E48</f>
+        <f>+FORMATO!D48</f>
         <v>0</v>
       </c>
       <c r="T31" s="523">
@@ -24152,16 +24152,16 @@
       <c r="B32" s="623"/>
       <c r="C32" s="623"/>
       <c r="D32" s="623"/>
-      <c r="E32" s="835" t="s">
+      <c r="E32" s="827" t="s">
         <v>232</v>
       </c>
-      <c r="F32" s="836"/>
-      <c r="G32" s="836"/>
-      <c r="H32" s="837"/>
-      <c r="I32" s="838" t="s">
+      <c r="F32" s="828"/>
+      <c r="G32" s="828"/>
+      <c r="H32" s="829"/>
+      <c r="I32" s="863" t="s">
         <v>456</v>
       </c>
-      <c r="J32" s="839"/>
+      <c r="J32" s="864"/>
       <c r="K32" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$32),0),FIXED(($W$32),1))</f>
         <v>#DIV/0!</v>
@@ -24178,7 +24178,7 @@
         <v>2</v>
       </c>
       <c r="S32" s="665">
-        <f>+FORMATO!E50</f>
+        <f>+FORMATO!D50</f>
         <v>0</v>
       </c>
       <c r="T32" s="523">
@@ -24212,16 +24212,16 @@
       <c r="B33" s="623"/>
       <c r="C33" s="623"/>
       <c r="D33" s="623"/>
-      <c r="E33" s="835" t="s">
+      <c r="E33" s="827" t="s">
         <v>238</v>
       </c>
-      <c r="F33" s="836"/>
-      <c r="G33" s="836"/>
-      <c r="H33" s="837"/>
-      <c r="I33" s="840" t="s">
+      <c r="F33" s="828"/>
+      <c r="G33" s="828"/>
+      <c r="H33" s="829"/>
+      <c r="I33" s="859" t="s">
         <v>458</v>
       </c>
-      <c r="J33" s="841"/>
+      <c r="J33" s="860"/>
       <c r="K33" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$33),0),FIXED(($W$33),1))</f>
         <v>#DIV/0!</v>
@@ -24238,7 +24238,7 @@
         <v>0.85</v>
       </c>
       <c r="S33" s="665">
-        <f>+FORMATO!E51</f>
+        <f>+FORMATO!D51</f>
         <v>0</v>
       </c>
       <c r="T33" s="523">
@@ -24264,16 +24264,16 @@
       <c r="B34" s="623"/>
       <c r="C34" s="623"/>
       <c r="D34" s="623"/>
-      <c r="E34" s="835" t="s">
+      <c r="E34" s="827" t="s">
         <v>418</v>
       </c>
-      <c r="F34" s="836"/>
-      <c r="G34" s="836"/>
-      <c r="H34" s="837"/>
-      <c r="I34" s="840" t="s">
+      <c r="F34" s="828"/>
+      <c r="G34" s="828"/>
+      <c r="H34" s="829"/>
+      <c r="I34" s="859" t="s">
         <v>459</v>
       </c>
-      <c r="J34" s="841"/>
+      <c r="J34" s="860"/>
       <c r="K34" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$34),0),FIXED(($W$34),1))</f>
         <v>#DIV/0!</v>
@@ -24290,7 +24290,7 @@
         <v>0.42499999999999999</v>
       </c>
       <c r="S34" s="665">
-        <f>+FORMATO!E52</f>
+        <f>+FORMATO!D52</f>
         <v>0</v>
       </c>
       <c r="T34" s="523">
@@ -24320,16 +24320,16 @@
       <c r="B35" s="623"/>
       <c r="C35" s="623"/>
       <c r="D35" s="623"/>
-      <c r="E35" s="835" t="s">
+      <c r="E35" s="827" t="s">
         <v>239</v>
       </c>
-      <c r="F35" s="836"/>
-      <c r="G35" s="836"/>
-      <c r="H35" s="837"/>
-      <c r="I35" s="840" t="s">
+      <c r="F35" s="828"/>
+      <c r="G35" s="828"/>
+      <c r="H35" s="829"/>
+      <c r="I35" s="859" t="s">
         <v>460</v>
       </c>
-      <c r="J35" s="841"/>
+      <c r="J35" s="860"/>
       <c r="K35" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$35),0),FIXED(($W$35),1))</f>
         <v>#DIV/0!</v>
@@ -24346,7 +24346,7 @@
         <v>0.25</v>
       </c>
       <c r="S35" s="665">
-        <f>+FORMATO!E53</f>
+        <f>+FORMATO!D53</f>
         <v>0</v>
       </c>
       <c r="T35" s="523">
@@ -24376,16 +24376,16 @@
       <c r="B36" s="623"/>
       <c r="C36" s="623"/>
       <c r="D36" s="623"/>
-      <c r="E36" s="835" t="s">
+      <c r="E36" s="827" t="s">
         <v>241</v>
       </c>
-      <c r="F36" s="836"/>
-      <c r="G36" s="836"/>
-      <c r="H36" s="837"/>
-      <c r="I36" s="840" t="s">
+      <c r="F36" s="828"/>
+      <c r="G36" s="828"/>
+      <c r="H36" s="829"/>
+      <c r="I36" s="859" t="s">
         <v>461</v>
       </c>
-      <c r="J36" s="841"/>
+      <c r="J36" s="860"/>
       <c r="K36" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$36),0),FIXED(($W$36),1))</f>
         <v>#DIV/0!</v>
@@ -24402,7 +24402,7 @@
         <v>0.15</v>
       </c>
       <c r="S36" s="665">
-        <f>+FORMATO!E54</f>
+        <f>+FORMATO!D54</f>
         <v>0</v>
       </c>
       <c r="T36" s="523">
@@ -24431,16 +24431,16 @@
       <c r="B37" s="623"/>
       <c r="C37" s="623"/>
       <c r="D37" s="623"/>
-      <c r="E37" s="835" t="s">
+      <c r="E37" s="827" t="s">
         <v>240</v>
       </c>
-      <c r="F37" s="836"/>
-      <c r="G37" s="836"/>
-      <c r="H37" s="837"/>
-      <c r="I37" s="840" t="s">
+      <c r="F37" s="828"/>
+      <c r="G37" s="828"/>
+      <c r="H37" s="829"/>
+      <c r="I37" s="859" t="s">
         <v>462</v>
       </c>
-      <c r="J37" s="841"/>
+      <c r="J37" s="860"/>
       <c r="K37" s="618" t="e">
         <f>IF($I$66="Método A",FIXED(($W$37),0),FIXED(($W$37),1))</f>
         <v>#DIV/0!</v>
@@ -24457,7 +24457,7 @@
         <v>0.106</v>
       </c>
       <c r="S37" s="665">
-        <f>+FORMATO!E55</f>
+        <f>+FORMATO!D55</f>
         <v>0</v>
       </c>
       <c r="T37" s="523">
@@ -24486,16 +24486,16 @@
       <c r="B38" s="623"/>
       <c r="C38" s="623"/>
       <c r="D38" s="623"/>
-      <c r="E38" s="892" t="s">
+      <c r="E38" s="830" t="s">
         <v>242</v>
       </c>
-      <c r="F38" s="893"/>
-      <c r="G38" s="893"/>
-      <c r="H38" s="894"/>
-      <c r="I38" s="898" t="s">
+      <c r="F38" s="831"/>
+      <c r="G38" s="831"/>
+      <c r="H38" s="832"/>
+      <c r="I38" s="838" t="s">
         <v>463</v>
       </c>
-      <c r="J38" s="899"/>
+      <c r="J38" s="839"/>
       <c r="K38" s="317" t="e">
         <f>IF($I$66="Método A",FIXED(($W$38),0),FIXED(($W$38),1))</f>
         <v>#DIV/0!</v>
@@ -24512,7 +24512,7 @@
         <v>7.4999999999999997E-2</v>
       </c>
       <c r="S38" s="665">
-        <f>+FORMATO!E56</f>
+        <f>+FORMATO!D56</f>
         <v>0</v>
       </c>
       <c r="T38" s="523">
@@ -24562,7 +24562,7 @@
         <v>0.01</v>
       </c>
       <c r="S39" s="665">
-        <f>+FORMATO!E57</f>
+        <f>+FORMATO!D57</f>
         <v>0</v>
       </c>
       <c r="T39" s="523" t="b">
@@ -24628,12 +24628,12 @@
       <c r="N41" s="313"/>
       <c r="O41" s="570"/>
       <c r="P41" s="570"/>
-      <c r="Q41" s="843" t="s">
+      <c r="Q41" s="880" t="s">
         <v>420</v>
       </c>
-      <c r="R41" s="844"/>
-      <c r="S41" s="844"/>
-      <c r="T41" s="845"/>
+      <c r="R41" s="881"/>
+      <c r="S41" s="881"/>
+      <c r="T41" s="882"/>
       <c r="AA41" s="513"/>
       <c r="AB41" s="513"/>
       <c r="AC41" s="513"/>
@@ -24656,10 +24656,10 @@
       <c r="N42" s="313"/>
       <c r="O42" s="570"/>
       <c r="P42" s="570"/>
-      <c r="Q42" s="846"/>
-      <c r="R42" s="847"/>
-      <c r="S42" s="847"/>
-      <c r="T42" s="848"/>
+      <c r="Q42" s="883"/>
+      <c r="R42" s="884"/>
+      <c r="S42" s="884"/>
+      <c r="T42" s="885"/>
       <c r="U42" s="620"/>
       <c r="V42" s="620"/>
       <c r="AA42" s="513"/>
@@ -24684,10 +24684,10 @@
       <c r="N43" s="313"/>
       <c r="O43" s="570"/>
       <c r="P43" s="570"/>
-      <c r="Q43" s="849" t="s">
+      <c r="Q43" s="886" t="s">
         <v>34</v>
       </c>
-      <c r="R43" s="851" t="e">
+      <c r="R43" s="888" t="e">
         <f>$V$31</f>
         <v>#DIV/0!</v>
       </c>
@@ -24722,8 +24722,8 @@
       <c r="N44" s="313"/>
       <c r="O44" s="570"/>
       <c r="P44" s="570"/>
-      <c r="Q44" s="850"/>
-      <c r="R44" s="852"/>
+      <c r="Q44" s="887"/>
+      <c r="R44" s="889"/>
       <c r="S44" s="311" t="s">
         <v>36</v>
       </c>
@@ -24757,10 +24757,10 @@
       <c r="N45" s="313"/>
       <c r="O45" s="570"/>
       <c r="P45" s="570"/>
-      <c r="Q45" s="853" t="s">
+      <c r="Q45" s="890" t="s">
         <v>37</v>
       </c>
-      <c r="R45" s="855" t="e">
+      <c r="R45" s="892" t="e">
         <f>100-(R43+R48)</f>
         <v>#DIV/0!</v>
       </c>
@@ -24798,8 +24798,8 @@
       <c r="N46" s="313"/>
       <c r="O46" s="570"/>
       <c r="P46" s="570"/>
-      <c r="Q46" s="854"/>
-      <c r="R46" s="856"/>
+      <c r="Q46" s="891"/>
+      <c r="R46" s="893"/>
       <c r="S46" s="311" t="s">
         <v>38</v>
       </c>
@@ -24833,8 +24833,8 @@
       <c r="N47" s="313"/>
       <c r="O47" s="570"/>
       <c r="P47" s="570"/>
-      <c r="Q47" s="850"/>
-      <c r="R47" s="852"/>
+      <c r="Q47" s="887"/>
+      <c r="R47" s="889"/>
       <c r="S47" s="311" t="s">
         <v>36</v>
       </c>
@@ -25435,12 +25435,12 @@
       <c r="F66" s="306"/>
       <c r="G66" s="306"/>
       <c r="H66" s="306"/>
-      <c r="I66" s="888" t="str">
+      <c r="I66" s="834" t="str">
         <f>+R2</f>
         <v>-</v>
       </c>
-      <c r="J66" s="888"/>
-      <c r="K66" s="888"/>
+      <c r="J66" s="834"/>
+      <c r="K66" s="834"/>
       <c r="L66" s="421"/>
       <c r="M66" s="421"/>
       <c r="N66" s="545"/>
@@ -25472,11 +25472,11 @@
       <c r="F67" s="306"/>
       <c r="G67" s="306"/>
       <c r="H67" s="306"/>
-      <c r="I67" s="888" t="s">
+      <c r="I67" s="834" t="s">
         <v>442</v>
       </c>
-      <c r="J67" s="888"/>
-      <c r="K67" s="888"/>
+      <c r="J67" s="834"/>
+      <c r="K67" s="834"/>
       <c r="L67" s="421"/>
       <c r="M67" s="421"/>
       <c r="N67" s="545"/>
@@ -25508,11 +25508,11 @@
       <c r="F68" s="546"/>
       <c r="G68" s="546"/>
       <c r="H68" s="546"/>
-      <c r="I68" s="888" t="s">
+      <c r="I68" s="834" t="s">
         <v>442</v>
       </c>
-      <c r="J68" s="888"/>
-      <c r="K68" s="888"/>
+      <c r="J68" s="834"/>
+      <c r="K68" s="834"/>
       <c r="L68" s="421"/>
       <c r="M68" s="421"/>
       <c r="N68" s="545"/>
@@ -25544,11 +25544,11 @@
       <c r="F69" s="546"/>
       <c r="G69" s="546"/>
       <c r="H69" s="546"/>
-      <c r="I69" s="842" t="s">
+      <c r="I69" s="833" t="s">
         <v>252</v>
       </c>
-      <c r="J69" s="842"/>
-      <c r="K69" s="842"/>
+      <c r="J69" s="833"/>
+      <c r="K69" s="833"/>
       <c r="L69" s="421"/>
       <c r="M69" s="421"/>
       <c r="N69" s="545"/>
@@ -25580,11 +25580,11 @@
       <c r="F70" s="546"/>
       <c r="G70" s="546"/>
       <c r="H70" s="546"/>
-      <c r="I70" s="888" t="s">
+      <c r="I70" s="834" t="s">
         <v>442</v>
       </c>
-      <c r="J70" s="888"/>
-      <c r="K70" s="888"/>
+      <c r="J70" s="834"/>
+      <c r="K70" s="834"/>
       <c r="L70" s="421"/>
       <c r="M70" s="421"/>
       <c r="N70" s="545"/>
@@ -25616,11 +25616,11 @@
       <c r="F71" s="546"/>
       <c r="G71" s="546"/>
       <c r="H71" s="546"/>
-      <c r="I71" s="842" t="s">
+      <c r="I71" s="833" t="s">
         <v>252</v>
       </c>
-      <c r="J71" s="842"/>
-      <c r="K71" s="842"/>
+      <c r="J71" s="833"/>
+      <c r="K71" s="833"/>
       <c r="L71" s="421"/>
       <c r="M71" s="421"/>
       <c r="N71" s="545"/>
@@ -25652,11 +25652,11 @@
       <c r="F72" s="306"/>
       <c r="G72" s="306"/>
       <c r="H72" s="306"/>
-      <c r="I72" s="895" t="s">
+      <c r="I72" s="835" t="s">
         <v>442</v>
       </c>
-      <c r="J72" s="896"/>
-      <c r="K72" s="897"/>
+      <c r="J72" s="836"/>
+      <c r="K72" s="837"/>
       <c r="L72" s="319"/>
       <c r="M72" s="319"/>
       <c r="N72" s="547"/>
@@ -25752,14 +25752,14 @@
       <c r="E75" s="306"/>
       <c r="F75" s="306"/>
       <c r="H75" s="306"/>
-      <c r="I75" s="842"/>
-      <c r="J75" s="842"/>
-      <c r="K75" s="842"/>
-      <c r="L75" s="827">
+      <c r="I75" s="833"/>
+      <c r="J75" s="833"/>
+      <c r="K75" s="833"/>
+      <c r="L75" s="894">
         <v>0</v>
       </c>
-      <c r="M75" s="828"/>
-      <c r="N75" s="829"/>
+      <c r="M75" s="895"/>
+      <c r="N75" s="896"/>
       <c r="O75" s="570"/>
       <c r="P75" s="570"/>
       <c r="Q75" s="424"/>
@@ -25787,11 +25787,11 @@
       <c r="E76" s="306"/>
       <c r="F76" s="306"/>
       <c r="H76" s="306"/>
-      <c r="I76" s="888" t="s">
+      <c r="I76" s="834" t="s">
         <v>442</v>
       </c>
-      <c r="J76" s="888"/>
-      <c r="K76" s="888"/>
+      <c r="J76" s="834"/>
+      <c r="K76" s="834"/>
       <c r="L76" s="306"/>
       <c r="M76" s="306"/>
       <c r="N76" s="552"/>
@@ -25822,12 +25822,12 @@
       <c r="E77" s="306"/>
       <c r="F77" s="306"/>
       <c r="H77" s="306"/>
-      <c r="I77" s="889">
+      <c r="I77" s="841">
         <f>+FORMATO!H19</f>
         <v>0</v>
       </c>
-      <c r="J77" s="842"/>
-      <c r="K77" s="842"/>
+      <c r="J77" s="833"/>
+      <c r="K77" s="833"/>
       <c r="L77" s="306"/>
       <c r="M77" s="306"/>
       <c r="N77" s="552"/>
@@ -25858,12 +25858,12 @@
       <c r="E78" s="306"/>
       <c r="F78" s="306"/>
       <c r="H78" s="306"/>
-      <c r="I78" s="888">
+      <c r="I78" s="834">
         <f>+FORMATO!H20</f>
         <v>0</v>
       </c>
-      <c r="J78" s="888"/>
-      <c r="K78" s="888"/>
+      <c r="J78" s="834"/>
+      <c r="K78" s="834"/>
       <c r="L78" s="306"/>
       <c r="M78" s="306"/>
       <c r="N78" s="552"/>
@@ -25951,22 +25951,22 @@
       <c r="AD80" s="513"/>
     </row>
     <row r="81" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="891" t="s">
+      <c r="A81" s="843" t="s">
         <v>568</v>
       </c>
-      <c r="B81" s="891"/>
-      <c r="C81" s="891"/>
-      <c r="D81" s="891"/>
-      <c r="E81" s="891"/>
-      <c r="F81" s="891"/>
-      <c r="G81" s="891"/>
-      <c r="H81" s="891"/>
-      <c r="I81" s="891"/>
-      <c r="J81" s="891"/>
-      <c r="K81" s="891"/>
-      <c r="L81" s="891"/>
-      <c r="M81" s="891"/>
-      <c r="N81" s="891"/>
+      <c r="B81" s="843"/>
+      <c r="C81" s="843"/>
+      <c r="D81" s="843"/>
+      <c r="E81" s="843"/>
+      <c r="F81" s="843"/>
+      <c r="G81" s="843"/>
+      <c r="H81" s="843"/>
+      <c r="I81" s="843"/>
+      <c r="J81" s="843"/>
+      <c r="K81" s="843"/>
+      <c r="L81" s="843"/>
+      <c r="M81" s="843"/>
+      <c r="N81" s="843"/>
       <c r="O81" s="426"/>
       <c r="P81" s="426"/>
       <c r="Q81" s="424"/>
@@ -25985,22 +25985,22 @@
       <c r="AD81" s="513"/>
     </row>
     <row r="82" spans="1:30" ht="35.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="890" t="s">
+      <c r="A82" s="842" t="s">
         <v>569</v>
       </c>
-      <c r="B82" s="890"/>
-      <c r="C82" s="890"/>
-      <c r="D82" s="890"/>
-      <c r="E82" s="890"/>
-      <c r="F82" s="890"/>
-      <c r="G82" s="890"/>
-      <c r="H82" s="890"/>
-      <c r="I82" s="890"/>
-      <c r="J82" s="890"/>
-      <c r="K82" s="890"/>
-      <c r="L82" s="890"/>
-      <c r="M82" s="890"/>
-      <c r="N82" s="890"/>
+      <c r="B82" s="842"/>
+      <c r="C82" s="842"/>
+      <c r="D82" s="842"/>
+      <c r="E82" s="842"/>
+      <c r="F82" s="842"/>
+      <c r="G82" s="842"/>
+      <c r="H82" s="842"/>
+      <c r="I82" s="842"/>
+      <c r="J82" s="842"/>
+      <c r="K82" s="842"/>
+      <c r="L82" s="842"/>
+      <c r="M82" s="842"/>
+      <c r="N82" s="842"/>
       <c r="Q82" s="424"/>
       <c r="R82" s="519"/>
       <c r="S82" s="519"/>
@@ -26017,22 +26017,22 @@
       <c r="AD82" s="513"/>
     </row>
     <row r="83" spans="1:30" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="890" t="s">
+      <c r="A83" s="842" t="s">
         <v>570</v>
       </c>
-      <c r="B83" s="890"/>
-      <c r="C83" s="890"/>
-      <c r="D83" s="890"/>
-      <c r="E83" s="890"/>
-      <c r="F83" s="890"/>
-      <c r="G83" s="890"/>
-      <c r="H83" s="890"/>
-      <c r="I83" s="890"/>
-      <c r="J83" s="890"/>
-      <c r="K83" s="890"/>
-      <c r="L83" s="890"/>
-      <c r="M83" s="890"/>
-      <c r="N83" s="890"/>
+      <c r="B83" s="842"/>
+      <c r="C83" s="842"/>
+      <c r="D83" s="842"/>
+      <c r="E83" s="842"/>
+      <c r="F83" s="842"/>
+      <c r="G83" s="842"/>
+      <c r="H83" s="842"/>
+      <c r="I83" s="842"/>
+      <c r="J83" s="842"/>
+      <c r="K83" s="842"/>
+      <c r="L83" s="842"/>
+      <c r="M83" s="842"/>
+      <c r="N83" s="842"/>
       <c r="O83" s="428"/>
       <c r="P83" s="428"/>
       <c r="AA83" s="513"/>
@@ -26041,44 +26041,44 @@
       <c r="AD83" s="513"/>
     </row>
     <row r="84" spans="1:30" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="890" t="s">
+      <c r="A84" s="842" t="s">
         <v>571</v>
       </c>
-      <c r="B84" s="890"/>
-      <c r="C84" s="890"/>
-      <c r="D84" s="890"/>
-      <c r="E84" s="890"/>
-      <c r="F84" s="890"/>
-      <c r="G84" s="890"/>
-      <c r="H84" s="890"/>
-      <c r="I84" s="890"/>
-      <c r="J84" s="890"/>
-      <c r="K84" s="890"/>
-      <c r="L84" s="890"/>
-      <c r="M84" s="890"/>
-      <c r="N84" s="890"/>
+      <c r="B84" s="842"/>
+      <c r="C84" s="842"/>
+      <c r="D84" s="842"/>
+      <c r="E84" s="842"/>
+      <c r="F84" s="842"/>
+      <c r="G84" s="842"/>
+      <c r="H84" s="842"/>
+      <c r="I84" s="842"/>
+      <c r="J84" s="842"/>
+      <c r="K84" s="842"/>
+      <c r="L84" s="842"/>
+      <c r="M84" s="842"/>
+      <c r="N84" s="842"/>
       <c r="AA84" s="513"/>
       <c r="AB84" s="513"/>
       <c r="AC84" s="513"/>
       <c r="AD84" s="513"/>
     </row>
     <row r="85" spans="1:30" ht="25.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="887" t="s">
+      <c r="A85" s="840" t="s">
         <v>572</v>
       </c>
-      <c r="B85" s="887"/>
-      <c r="C85" s="887"/>
-      <c r="D85" s="887"/>
-      <c r="E85" s="887"/>
-      <c r="F85" s="887"/>
-      <c r="G85" s="887"/>
-      <c r="H85" s="887"/>
-      <c r="I85" s="887"/>
-      <c r="J85" s="887"/>
-      <c r="K85" s="887"/>
-      <c r="L85" s="887"/>
-      <c r="M85" s="887"/>
-      <c r="N85" s="887"/>
+      <c r="B85" s="840"/>
+      <c r="C85" s="840"/>
+      <c r="D85" s="840"/>
+      <c r="E85" s="840"/>
+      <c r="F85" s="840"/>
+      <c r="G85" s="840"/>
+      <c r="H85" s="840"/>
+      <c r="I85" s="840"/>
+      <c r="J85" s="840"/>
+      <c r="K85" s="840"/>
+      <c r="L85" s="840"/>
+      <c r="M85" s="840"/>
+      <c r="N85" s="840"/>
       <c r="AA85" s="513"/>
       <c r="AB85" s="513"/>
       <c r="AC85" s="513"/>
@@ -26254,57 +26254,6 @@
   </protectedRanges>
   <dataConsolidate/>
   <mergeCells count="67">
-    <mergeCell ref="E37:H37"/>
-    <mergeCell ref="E38:H38"/>
-    <mergeCell ref="I75:K75"/>
-    <mergeCell ref="I66:K66"/>
-    <mergeCell ref="I67:K67"/>
-    <mergeCell ref="I72:K72"/>
-    <mergeCell ref="I68:K68"/>
-    <mergeCell ref="I69:K69"/>
-    <mergeCell ref="I70:K70"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="A85:N85"/>
-    <mergeCell ref="I76:K76"/>
-    <mergeCell ref="I77:K77"/>
-    <mergeCell ref="I78:K78"/>
-    <mergeCell ref="A83:N83"/>
-    <mergeCell ref="A81:N81"/>
-    <mergeCell ref="A82:N82"/>
-    <mergeCell ref="A84:N84"/>
-    <mergeCell ref="Q5:V5"/>
-    <mergeCell ref="A7:N7"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="A14:N14"/>
-    <mergeCell ref="A15:N15"/>
-    <mergeCell ref="A8:N8"/>
-    <mergeCell ref="Q16:V16"/>
-    <mergeCell ref="Q11:V11"/>
-    <mergeCell ref="C10:K10"/>
-    <mergeCell ref="C12:K12"/>
-    <mergeCell ref="C11:K11"/>
-    <mergeCell ref="C9:K9"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="E32:H32"/>
-    <mergeCell ref="E33:H33"/>
-    <mergeCell ref="X17:AA17"/>
-    <mergeCell ref="K23:K24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="E23:J23"/>
-    <mergeCell ref="E24:H24"/>
-    <mergeCell ref="E25:H25"/>
-    <mergeCell ref="E26:H26"/>
-    <mergeCell ref="Q41:T42"/>
-    <mergeCell ref="Q43:Q44"/>
-    <mergeCell ref="R43:R44"/>
-    <mergeCell ref="Q45:Q47"/>
-    <mergeCell ref="R45:R47"/>
     <mergeCell ref="L75:N75"/>
     <mergeCell ref="E27:H27"/>
     <mergeCell ref="I27:J27"/>
@@ -26321,6 +26270,57 @@
     <mergeCell ref="I35:J35"/>
     <mergeCell ref="I71:K71"/>
     <mergeCell ref="I37:J37"/>
+    <mergeCell ref="Q41:T42"/>
+    <mergeCell ref="Q43:Q44"/>
+    <mergeCell ref="R43:R44"/>
+    <mergeCell ref="Q45:Q47"/>
+    <mergeCell ref="R45:R47"/>
+    <mergeCell ref="X17:AA17"/>
+    <mergeCell ref="K23:K24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="E23:J23"/>
+    <mergeCell ref="E24:H24"/>
+    <mergeCell ref="E25:H25"/>
+    <mergeCell ref="E26:H26"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="E32:H32"/>
+    <mergeCell ref="E33:H33"/>
+    <mergeCell ref="Q5:V5"/>
+    <mergeCell ref="A7:N7"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="A14:N14"/>
+    <mergeCell ref="A15:N15"/>
+    <mergeCell ref="A8:N8"/>
+    <mergeCell ref="Q16:V16"/>
+    <mergeCell ref="Q11:V11"/>
+    <mergeCell ref="C10:K10"/>
+    <mergeCell ref="C12:K12"/>
+    <mergeCell ref="C11:K11"/>
+    <mergeCell ref="C9:K9"/>
+    <mergeCell ref="A85:N85"/>
+    <mergeCell ref="I76:K76"/>
+    <mergeCell ref="I77:K77"/>
+    <mergeCell ref="I78:K78"/>
+    <mergeCell ref="A83:N83"/>
+    <mergeCell ref="A81:N81"/>
+    <mergeCell ref="A82:N82"/>
+    <mergeCell ref="A84:N84"/>
+    <mergeCell ref="E37:H37"/>
+    <mergeCell ref="E38:H38"/>
+    <mergeCell ref="I75:K75"/>
+    <mergeCell ref="I66:K66"/>
+    <mergeCell ref="I67:K67"/>
+    <mergeCell ref="I72:K72"/>
+    <mergeCell ref="I68:K68"/>
+    <mergeCell ref="I69:K69"/>
+    <mergeCell ref="I70:K70"/>
+    <mergeCell ref="I38:J38"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <conditionalFormatting sqref="AA24">
@@ -32990,35 +32990,35 @@
       <c r="K7" s="150"/>
     </row>
     <row r="8" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="936" t="s">
+      <c r="A8" s="958" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="936"/>
-      <c r="C8" s="936"/>
-      <c r="D8" s="936"/>
-      <c r="E8" s="936"/>
-      <c r="F8" s="936"/>
-      <c r="G8" s="936"/>
-      <c r="H8" s="936"/>
-      <c r="I8" s="936"/>
-      <c r="J8" s="936"/>
-      <c r="K8" s="936"/>
+      <c r="B8" s="958"/>
+      <c r="C8" s="958"/>
+      <c r="D8" s="958"/>
+      <c r="E8" s="958"/>
+      <c r="F8" s="958"/>
+      <c r="G8" s="958"/>
+      <c r="H8" s="958"/>
+      <c r="I8" s="958"/>
+      <c r="J8" s="958"/>
+      <c r="K8" s="958"/>
     </row>
     <row r="9" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="937">
+      <c r="A9" s="959">
         <f>+K13</f>
         <v>10</v>
       </c>
-      <c r="B9" s="937"/>
-      <c r="C9" s="937"/>
-      <c r="D9" s="937"/>
-      <c r="E9" s="937"/>
-      <c r="F9" s="937"/>
-      <c r="G9" s="937"/>
-      <c r="H9" s="937"/>
-      <c r="I9" s="937"/>
-      <c r="J9" s="937"/>
-      <c r="K9" s="937"/>
+      <c r="B9" s="959"/>
+      <c r="C9" s="959"/>
+      <c r="D9" s="959"/>
+      <c r="E9" s="959"/>
+      <c r="F9" s="959"/>
+      <c r="G9" s="959"/>
+      <c r="H9" s="959"/>
+      <c r="I9" s="959"/>
+      <c r="J9" s="959"/>
+      <c r="K9" s="959"/>
       <c r="O9" s="151"/>
     </row>
     <row r="10" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -33041,15 +33041,15 @@
       <c r="B11" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="938">
+      <c r="C11" s="960">
         <f>+A.Granul!F10</f>
         <v>0</v>
       </c>
-      <c r="D11" s="938"/>
-      <c r="E11" s="938"/>
-      <c r="F11" s="938"/>
-      <c r="G11" s="938"/>
-      <c r="H11" s="938"/>
+      <c r="D11" s="960"/>
+      <c r="E11" s="960"/>
+      <c r="F11" s="960"/>
+      <c r="G11" s="960"/>
+      <c r="H11" s="960"/>
       <c r="I11" s="153" t="s">
         <v>31</v>
       </c>
@@ -33070,15 +33070,15 @@
       <c r="B12" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="938">
+      <c r="C12" s="960">
         <f>+A.Granul!F11</f>
         <v>0</v>
       </c>
-      <c r="D12" s="938"/>
-      <c r="E12" s="938"/>
-      <c r="F12" s="938"/>
-      <c r="G12" s="938"/>
-      <c r="H12" s="938"/>
+      <c r="D12" s="960"/>
+      <c r="E12" s="960"/>
+      <c r="F12" s="960"/>
+      <c r="G12" s="960"/>
+      <c r="H12" s="960"/>
       <c r="I12" s="15" t="s">
         <v>19</v>
       </c>
@@ -33103,15 +33103,15 @@
       <c r="B13" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="938">
+      <c r="C13" s="960">
         <f>+A.Granul!F12</f>
         <v>0</v>
       </c>
-      <c r="D13" s="938"/>
-      <c r="E13" s="938"/>
-      <c r="F13" s="938"/>
-      <c r="G13" s="938"/>
-      <c r="H13" s="938"/>
+      <c r="D13" s="960"/>
+      <c r="E13" s="960"/>
+      <c r="F13" s="960"/>
+      <c r="G13" s="960"/>
+      <c r="H13" s="960"/>
       <c r="I13" s="15" t="s">
         <v>20</v>
       </c>
@@ -33125,8 +33125,8 @@
       <c r="M13" s="156"/>
       <c r="P13" s="159"/>
       <c r="Q13" s="159"/>
-      <c r="R13" s="935"/>
-      <c r="S13" s="935"/>
+      <c r="R13" s="957"/>
+      <c r="S13" s="957"/>
     </row>
     <row r="14" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
@@ -33148,19 +33148,19 @@
       <c r="S14" s="164"/>
     </row>
     <row r="15" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="940" t="s">
+      <c r="A15" s="943" t="s">
         <v>171</v>
       </c>
-      <c r="B15" s="941"/>
-      <c r="C15" s="941"/>
-      <c r="D15" s="941"/>
-      <c r="E15" s="941"/>
-      <c r="F15" s="941"/>
-      <c r="G15" s="941"/>
-      <c r="H15" s="941"/>
-      <c r="I15" s="941"/>
-      <c r="J15" s="941"/>
-      <c r="K15" s="942"/>
+      <c r="B15" s="944"/>
+      <c r="C15" s="944"/>
+      <c r="D15" s="944"/>
+      <c r="E15" s="944"/>
+      <c r="F15" s="944"/>
+      <c r="G15" s="944"/>
+      <c r="H15" s="944"/>
+      <c r="I15" s="944"/>
+      <c r="J15" s="944"/>
+      <c r="K15" s="945"/>
       <c r="L15" s="156"/>
       <c r="M15" s="156"/>
       <c r="P15" s="159"/>
@@ -33169,19 +33169,19 @@
       <c r="S15" s="164"/>
     </row>
     <row r="16" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="943" t="s">
+      <c r="A16" s="946" t="s">
         <v>191</v>
       </c>
-      <c r="B16" s="944"/>
-      <c r="C16" s="944"/>
-      <c r="D16" s="944"/>
-      <c r="E16" s="944"/>
-      <c r="F16" s="944"/>
-      <c r="G16" s="944"/>
-      <c r="H16" s="944"/>
-      <c r="I16" s="944"/>
-      <c r="J16" s="944"/>
-      <c r="K16" s="945"/>
+      <c r="B16" s="947"/>
+      <c r="C16" s="947"/>
+      <c r="D16" s="947"/>
+      <c r="E16" s="947"/>
+      <c r="F16" s="947"/>
+      <c r="G16" s="947"/>
+      <c r="H16" s="947"/>
+      <c r="I16" s="947"/>
+      <c r="J16" s="947"/>
+      <c r="K16" s="948"/>
       <c r="L16" s="156"/>
       <c r="M16" s="156"/>
       <c r="P16" s="159"/>
@@ -33209,19 +33209,19 @@
       <c r="S17" s="164"/>
     </row>
     <row r="18" spans="1:21" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="946" t="s">
+      <c r="A18" s="949" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="947"/>
-      <c r="C18" s="947"/>
-      <c r="D18" s="947"/>
-      <c r="E18" s="947"/>
-      <c r="F18" s="947"/>
-      <c r="G18" s="947"/>
-      <c r="H18" s="947"/>
-      <c r="I18" s="947"/>
-      <c r="J18" s="947"/>
-      <c r="K18" s="948"/>
+      <c r="B18" s="950"/>
+      <c r="C18" s="950"/>
+      <c r="D18" s="950"/>
+      <c r="E18" s="950"/>
+      <c r="F18" s="950"/>
+      <c r="G18" s="950"/>
+      <c r="H18" s="950"/>
+      <c r="I18" s="950"/>
+      <c r="J18" s="950"/>
+      <c r="K18" s="951"/>
       <c r="M18" s="156"/>
       <c r="P18" s="159"/>
       <c r="Q18" s="159"/>
@@ -33346,8 +33346,8 @@
     </row>
     <row r="23" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="176"/>
-      <c r="I23" s="949"/>
-      <c r="J23" s="949"/>
+      <c r="I23" s="952"/>
+      <c r="J23" s="952"/>
       <c r="K23" s="177"/>
       <c r="L23" s="156"/>
       <c r="M23" s="178"/>
@@ -33355,41 +33355,41 @@
     </row>
     <row r="24" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="180"/>
-      <c r="D24" s="950" t="s">
+      <c r="D24" s="953" t="s">
         <v>174</v>
       </c>
-      <c r="E24" s="951"/>
-      <c r="F24" s="951"/>
-      <c r="G24" s="952" t="s">
+      <c r="E24" s="954"/>
+      <c r="F24" s="954"/>
+      <c r="G24" s="955" t="s">
         <v>175</v>
       </c>
-      <c r="H24" s="953"/>
-      <c r="I24" s="954"/>
-      <c r="J24" s="954"/>
+      <c r="H24" s="956"/>
+      <c r="I24" s="940"/>
+      <c r="J24" s="940"/>
       <c r="K24" s="181"/>
       <c r="L24" s="156"/>
       <c r="M24" s="182"/>
-      <c r="O24" s="955" t="s">
+      <c r="O24" s="935" t="s">
         <v>174</v>
       </c>
-      <c r="P24" s="956"/>
+      <c r="P24" s="936"/>
       <c r="Q24" s="183" t="s">
         <v>173</v>
       </c>
-      <c r="R24" s="955" t="s">
+      <c r="R24" s="935" t="s">
         <v>175</v>
       </c>
-      <c r="S24" s="957"/>
+      <c r="S24" s="937"/>
       <c r="T24" s="183" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="25" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="180"/>
-      <c r="B25" s="958" t="s">
+      <c r="B25" s="938" t="s">
         <v>176</v>
       </c>
-      <c r="C25" s="959"/>
+      <c r="C25" s="939"/>
       <c r="D25" s="184" t="str">
         <f>IF($Q$24="NO","",O25)</f>
         <v/>
@@ -33410,8 +33410,8 @@
         <f>IF($T$24="NO","",S25)</f>
         <v/>
       </c>
-      <c r="I25" s="954"/>
-      <c r="J25" s="954"/>
+      <c r="I25" s="940"/>
+      <c r="J25" s="940"/>
       <c r="K25" s="181"/>
       <c r="L25" s="156"/>
       <c r="M25" s="182"/>
@@ -33460,8 +33460,8 @@
         <f>IF($T$24="NO","",S26)</f>
         <v/>
       </c>
-      <c r="I26" s="960"/>
-      <c r="J26" s="960"/>
+      <c r="I26" s="941"/>
+      <c r="J26" s="941"/>
       <c r="K26" s="194"/>
       <c r="L26" s="195"/>
       <c r="M26" s="182"/>
@@ -34239,19 +34239,19 @@
       <c r="Q49"/>
     </row>
     <row r="50" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="939" t="s">
+      <c r="A50" s="942" t="s">
         <v>192</v>
       </c>
-      <c r="B50" s="939"/>
-      <c r="C50" s="939"/>
-      <c r="D50" s="939"/>
-      <c r="E50" s="939"/>
-      <c r="F50" s="939"/>
-      <c r="G50" s="939"/>
-      <c r="H50" s="939"/>
-      <c r="I50" s="939"/>
-      <c r="J50" s="939"/>
-      <c r="K50" s="939"/>
+      <c r="B50" s="942"/>
+      <c r="C50" s="942"/>
+      <c r="D50" s="942"/>
+      <c r="E50" s="942"/>
+      <c r="F50" s="942"/>
+      <c r="G50" s="942"/>
+      <c r="H50" s="942"/>
+      <c r="I50" s="942"/>
+      <c r="J50" s="942"/>
+      <c r="K50" s="942"/>
     </row>
     <row r="51" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="52" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -34261,11 +34261,12 @@
     <protectedRange sqref="C11" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="19">
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="R13:S13"/>
+    <mergeCell ref="A8:K8"/>
+    <mergeCell ref="A9:K9"/>
+    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="C12:H12"/>
+    <mergeCell ref="C13:H13"/>
     <mergeCell ref="A50:K50"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A16:K16"/>
@@ -34274,12 +34275,11 @@
     <mergeCell ref="D24:F24"/>
     <mergeCell ref="G24:H24"/>
     <mergeCell ref="I24:J24"/>
-    <mergeCell ref="R13:S13"/>
-    <mergeCell ref="A8:K8"/>
-    <mergeCell ref="A9:K9"/>
-    <mergeCell ref="C11:H11"/>
-    <mergeCell ref="C12:H12"/>
-    <mergeCell ref="C13:H13"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="I26:J26"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q24 T24" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -34316,15 +34316,15 @@
       <c r="A1" s="94" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="961" t="s">
+      <c r="B1" s="980" t="s">
         <v>98</v>
       </c>
-      <c r="C1" s="961"/>
-      <c r="D1" s="961"/>
-      <c r="E1" s="961"/>
-      <c r="F1" s="961"/>
-      <c r="G1" s="961"/>
-      <c r="H1" s="961"/>
+      <c r="C1" s="980"/>
+      <c r="D1" s="980"/>
+      <c r="E1" s="980"/>
+      <c r="F1" s="980"/>
+      <c r="G1" s="980"/>
+      <c r="H1" s="980"/>
       <c r="I1" s="94"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -34462,29 +34462,29 @@
     </row>
     <row r="8" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="94"/>
-      <c r="B8" s="962" t="s">
+      <c r="B8" s="981" t="s">
         <v>110</v>
       </c>
-      <c r="C8" s="962"/>
-      <c r="D8" s="962"/>
+      <c r="C8" s="981"/>
+      <c r="D8" s="981"/>
       <c r="E8" s="103" t="s">
         <v>111</v>
       </c>
       <c r="F8" s="104" t="s">
         <v>112</v>
       </c>
-      <c r="G8" s="963" t="s">
+      <c r="G8" s="982" t="s">
         <v>113</v>
       </c>
-      <c r="H8" s="963"/>
+      <c r="H8" s="982"/>
       <c r="I8" s="94"/>
       <c r="L8" s="247" t="s">
         <v>114</v>
       </c>
-      <c r="M8" s="964" t="s">
+      <c r="M8" s="983" t="s">
         <v>115</v>
       </c>
-      <c r="N8" s="964"/>
+      <c r="N8" s="983"/>
       <c r="O8" s="248" t="s">
         <v>116</v>
       </c>
@@ -34497,13 +34497,13 @@
     </row>
     <row r="9" spans="1:17" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="94"/>
-      <c r="B9" s="965" t="s">
+      <c r="B9" s="984" t="s">
         <v>119</v>
       </c>
-      <c r="C9" s="967" t="s">
+      <c r="C9" s="986" t="s">
         <v>120</v>
       </c>
-      <c r="D9" s="969" t="s">
+      <c r="D9" s="988" t="s">
         <v>121</v>
       </c>
       <c r="E9" s="106" t="s">
@@ -34512,10 +34512,10 @@
       <c r="F9" s="107" t="s">
         <v>123</v>
       </c>
-      <c r="G9" s="970" t="s">
+      <c r="G9" s="989" t="s">
         <v>124</v>
       </c>
-      <c r="H9" s="971"/>
+      <c r="H9" s="990"/>
       <c r="I9" s="94"/>
       <c r="L9" s="249" t="e">
         <f>IF(AND(N_200&lt;50,(100-N_40)&gt;=0.5*(100-N_200),N_200&lt;5,CU&gt;=4,CC&gt;=1,CC&lt;=3),"GW","")</f>
@@ -34544,19 +34544,19 @@
     </row>
     <row r="10" spans="1:17" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="94"/>
-      <c r="B10" s="965"/>
-      <c r="C10" s="967"/>
-      <c r="D10" s="969"/>
+      <c r="B10" s="984"/>
+      <c r="C10" s="986"/>
+      <c r="D10" s="988"/>
       <c r="E10" s="108" t="s">
         <v>125</v>
       </c>
       <c r="F10" s="109" t="s">
         <v>126</v>
       </c>
-      <c r="G10" s="972" t="s">
+      <c r="G10" s="991" t="s">
         <v>127</v>
       </c>
-      <c r="H10" s="973"/>
+      <c r="H10" s="992"/>
       <c r="I10" s="94"/>
       <c r="L10" s="249" t="e">
         <f>IF(AND(N_200&lt;50,(100-N_40)&gt;=0.5*(100-N_200),N_200&lt;5,OR(CU&lt;4,CC&lt;1,CC&gt;3)),"GP","")</f>
@@ -34581,9 +34581,9 @@
     </row>
     <row r="11" spans="1:17" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="94"/>
-      <c r="B11" s="965"/>
-      <c r="C11" s="967"/>
-      <c r="D11" s="969" t="s">
+      <c r="B11" s="984"/>
+      <c r="C11" s="986"/>
+      <c r="D11" s="988" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="108" t="s">
@@ -34595,7 +34595,7 @@
       <c r="G11" s="111" t="s">
         <v>131</v>
       </c>
-      <c r="H11" s="974" t="s">
+      <c r="H11" s="993" t="s">
         <v>132</v>
       </c>
       <c r="I11" s="94"/>
@@ -34616,9 +34616,9 @@
     </row>
     <row r="12" spans="1:17" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="94"/>
-      <c r="B12" s="965"/>
-      <c r="C12" s="968"/>
-      <c r="D12" s="969"/>
+      <c r="B12" s="984"/>
+      <c r="C12" s="987"/>
+      <c r="D12" s="988"/>
       <c r="E12" s="112" t="s">
         <v>133</v>
       </c>
@@ -34628,7 +34628,7 @@
       <c r="G12" s="111" t="s">
         <v>135</v>
       </c>
-      <c r="H12" s="975"/>
+      <c r="H12" s="994"/>
       <c r="I12" s="94"/>
       <c r="L12" s="249" t="e">
         <f>IF(AND(N_200&lt;50,(100-N_40)&gt;=0.5*(100-N_200),N_200&gt;=12,IP&gt;=7,IP&gt;=0.73*(Ll-20)),"GC","")</f>
@@ -34644,11 +34644,11 @@
     </row>
     <row r="13" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="94"/>
-      <c r="B13" s="965"/>
-      <c r="C13" s="967" t="s">
+      <c r="B13" s="984"/>
+      <c r="C13" s="986" t="s">
         <v>136</v>
       </c>
-      <c r="D13" s="969" t="s">
+      <c r="D13" s="988" t="s">
         <v>137</v>
       </c>
       <c r="E13" s="113" t="s">
@@ -34657,10 +34657,10 @@
       <c r="F13" s="114" t="s">
         <v>139</v>
       </c>
-      <c r="G13" s="976" t="s">
+      <c r="G13" s="995" t="s">
         <v>140</v>
       </c>
-      <c r="H13" s="977"/>
+      <c r="H13" s="996"/>
       <c r="I13" s="94"/>
       <c r="L13" s="249" t="e">
         <f>IF(AND(N_200&lt;50,(100-N_40)&lt;0.5*(100-N_200),N_200&lt;5,CU&gt;=6,CC&gt;=1,CC&lt;=3),"SW","")</f>
@@ -34685,19 +34685,19 @@
     </row>
     <row r="14" spans="1:17" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="94"/>
-      <c r="B14" s="965"/>
-      <c r="C14" s="967"/>
-      <c r="D14" s="969"/>
+      <c r="B14" s="984"/>
+      <c r="C14" s="986"/>
+      <c r="D14" s="988"/>
       <c r="E14" s="113" t="s">
         <v>141</v>
       </c>
       <c r="F14" s="114" t="s">
         <v>142</v>
       </c>
-      <c r="G14" s="976" t="s">
+      <c r="G14" s="995" t="s">
         <v>143</v>
       </c>
-      <c r="H14" s="977"/>
+      <c r="H14" s="996"/>
       <c r="I14" s="94"/>
       <c r="L14" s="249" t="e">
         <f>IF(AND(N_200&lt;50,(100-N_40)&lt;0.5*(100-N_200),N_200&lt;5,OR(CU&lt;6,CC&lt;1,CC&gt;3)),"SP","")</f>
@@ -34722,9 +34722,9 @@
     </row>
     <row r="15" spans="1:17" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="94"/>
-      <c r="B15" s="965"/>
-      <c r="C15" s="967"/>
-      <c r="D15" s="969" t="s">
+      <c r="B15" s="984"/>
+      <c r="C15" s="986"/>
+      <c r="D15" s="988" t="s">
         <v>144</v>
       </c>
       <c r="E15" s="113" t="s">
@@ -34736,7 +34736,7 @@
       <c r="G15" s="116" t="s">
         <v>147</v>
       </c>
-      <c r="H15" s="980" t="s">
+      <c r="H15" s="963" t="s">
         <v>148</v>
       </c>
       <c r="I15" s="94"/>
@@ -34757,9 +34757,9 @@
     </row>
     <row r="16" spans="1:17" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="94"/>
-      <c r="B16" s="966"/>
-      <c r="C16" s="967"/>
-      <c r="D16" s="969"/>
+      <c r="B16" s="985"/>
+      <c r="C16" s="986"/>
+      <c r="D16" s="988"/>
       <c r="E16" s="117" t="s">
         <v>149</v>
       </c>
@@ -34769,7 +34769,7 @@
       <c r="G16" s="114" t="s">
         <v>151</v>
       </c>
-      <c r="H16" s="981"/>
+      <c r="H16" s="964"/>
       <c r="I16" s="94"/>
       <c r="L16" s="249" t="e">
         <f>IF(AND(N_200&lt;50,(100-N_40)&lt;0.5*(100-N_200),N_200&gt;=12,IP&gt;=7,IP&gt;=0.73*(Ll-20)),"SC","")</f>
@@ -34785,23 +34785,23 @@
     </row>
     <row r="17" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="94"/>
-      <c r="B17" s="982" t="s">
+      <c r="B17" s="965" t="s">
         <v>152</v>
       </c>
-      <c r="C17" s="985" t="s">
+      <c r="C17" s="968" t="s">
         <v>153</v>
       </c>
-      <c r="D17" s="986"/>
+      <c r="D17" s="969"/>
       <c r="E17" s="118" t="s">
         <v>154</v>
       </c>
       <c r="F17" s="119" t="s">
         <v>155</v>
       </c>
-      <c r="G17" s="991" t="s">
+      <c r="G17" s="974" t="s">
         <v>156</v>
       </c>
-      <c r="H17" s="992"/>
+      <c r="H17" s="975"/>
       <c r="I17" s="94"/>
       <c r="L17" s="249" t="e">
         <f>IF(AND(OR(L2="Inorganico"),N_200&gt;=50,Ll&lt;50,OR(IP&lt;4,AND(IP&lt;0.73*(Ll-20)))),"ML","")</f>
@@ -34817,17 +34817,17 @@
     </row>
     <row r="18" spans="1:16" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="94"/>
-      <c r="B18" s="983"/>
-      <c r="C18" s="987"/>
-      <c r="D18" s="988"/>
+      <c r="B18" s="966"/>
+      <c r="C18" s="970"/>
+      <c r="D18" s="971"/>
       <c r="E18" s="118" t="s">
         <v>157</v>
       </c>
       <c r="F18" s="119" t="s">
         <v>158</v>
       </c>
-      <c r="G18" s="993"/>
-      <c r="H18" s="994"/>
+      <c r="G18" s="976"/>
+      <c r="H18" s="977"/>
       <c r="I18" s="94"/>
       <c r="L18" s="249" t="e">
         <f>IF(AND(OR(L2="Inorganico"),N_200&gt;=50,Ll&lt;50,IP&gt;=7,IP&gt;=0.73*(Ll-20)),"CL","")</f>
@@ -34843,9 +34843,9 @@
     </row>
     <row r="19" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="94"/>
-      <c r="B19" s="983"/>
-      <c r="C19" s="989"/>
-      <c r="D19" s="990"/>
+      <c r="B19" s="966"/>
+      <c r="C19" s="972"/>
+      <c r="D19" s="973"/>
       <c r="E19" s="118" t="s">
         <v>159</v>
       </c>
@@ -34869,11 +34869,11 @@
     </row>
     <row r="20" spans="1:16" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="94"/>
-      <c r="B20" s="983"/>
-      <c r="C20" s="987" t="s">
+      <c r="B20" s="966"/>
+      <c r="C20" s="970" t="s">
         <v>161</v>
       </c>
-      <c r="D20" s="995"/>
+      <c r="D20" s="978"/>
       <c r="E20" s="122" t="s">
         <v>162</v>
       </c>
@@ -34897,9 +34897,9 @@
     </row>
     <row r="21" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="94"/>
-      <c r="B21" s="983"/>
-      <c r="C21" s="987"/>
-      <c r="D21" s="995"/>
+      <c r="B21" s="966"/>
+      <c r="C21" s="970"/>
+      <c r="D21" s="978"/>
       <c r="E21" s="122" t="s">
         <v>164</v>
       </c>
@@ -34923,9 +34923,9 @@
     </row>
     <row r="22" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="94"/>
-      <c r="B22" s="983"/>
-      <c r="C22" s="989"/>
-      <c r="D22" s="996"/>
+      <c r="B22" s="966"/>
+      <c r="C22" s="972"/>
+      <c r="D22" s="979"/>
       <c r="E22" s="124" t="s">
         <v>166</v>
       </c>
@@ -34949,11 +34949,11 @@
     </row>
     <row r="23" spans="1:16" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="94"/>
-      <c r="B23" s="983"/>
-      <c r="C23" s="985" t="s">
+      <c r="B23" s="966"/>
+      <c r="C23" s="968" t="s">
         <v>168</v>
       </c>
-      <c r="D23" s="986"/>
+      <c r="D23" s="969"/>
       <c r="E23" s="125" t="s">
         <v>169</v>
       </c>
@@ -34977,7 +34977,7 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="94"/>
-      <c r="B24" s="984"/>
+      <c r="B24" s="967"/>
       <c r="C24" s="127"/>
       <c r="D24" s="128"/>
       <c r="E24" s="129"/>
@@ -35073,10 +35073,10 @@
       <c r="F31" s="135"/>
     </row>
     <row r="32" spans="1:16" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="978" t="s">
+      <c r="A32" s="961" t="s">
         <v>200</v>
       </c>
-      <c r="B32" s="979"/>
+      <c r="B32" s="962"/>
       <c r="F32" s="135"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -35627,13 +35627,6 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="B17:B24"/>
-    <mergeCell ref="C17:D19"/>
-    <mergeCell ref="G17:H18"/>
-    <mergeCell ref="C20:D22"/>
-    <mergeCell ref="C23:D23"/>
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="G8:H8"/>
@@ -35650,6 +35643,13 @@
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="D15:D16"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="B17:B24"/>
+    <mergeCell ref="C17:D19"/>
+    <mergeCell ref="G17:H18"/>
+    <mergeCell ref="C20:D22"/>
+    <mergeCell ref="C23:D23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>